<commit_message>
magik num problem fikset
</commit_message>
<xml_diff>
--- a/MPLS_YAY/demo.xlsx
+++ b/MPLS_YAY/demo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yonat\Videos\INI\MPLS_YAY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473C2841-B1B3-4718-9250-752490D28F4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0D09B2A-28E6-4312-8424-B9A7EA6E3AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="65">
   <si>
     <t>site</t>
   </si>
@@ -225,6 +225,12 @@
   <si>
     <t>1337:40</t>
   </si>
+  <si>
+    <t>TEST</t>
+  </si>
+  <si>
+    <t>1337:50</t>
+  </si>
 </sst>
 </file>
 
@@ -329,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -379,6 +385,9 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -386,6 +395,329 @@
   <dxfs count="165">
     <dxf>
       <font>
+        <color theme="1"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -401,7 +733,6 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -421,7 +752,375 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -436,270 +1135,12 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="30" formatCode="@"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -788,6 +1229,309 @@
     <dxf>
       <font>
         <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -797,236 +1541,171 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
       </font>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1259,505 +1938,6 @@
     <dxf>
       <font>
         <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -1777,6 +1957,375 @@
     <dxf>
       <font>
         <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -1791,375 +2340,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2420,178 +2601,6 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <sz val="11"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <u val="none"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
@@ -2617,73 +2626,73 @@
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="brukernavn"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="passord"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="vty_lines"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="secret" dataDxfId="164"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="tacacs_key" dataDxfId="163"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="DHCP" dataDxfId="162"/>
-    <tableColumn id="10" xr3:uid="{B5E168AC-AF43-4637-AE64-122A38B00215}" name="dns_servers" dataDxfId="161"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="secret" dataDxfId="95"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="tacacs_key" dataDxfId="94"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="DHCP" dataDxfId="93"/>
+    <tableColumn id="10" xr3:uid="{B5E168AC-AF43-4637-AE64-122A38B00215}" name="dns_servers" dataDxfId="92"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="Tabell13192530" displayName="Tabell13192530" ref="A21:G22" headerRowDxfId="107" dataDxfId="106" totalsRowDxfId="105">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="29" xr:uid="{00000000-000C-0000-FFFF-FFFF09000000}" name="Tabell13192530" displayName="Tabell13192530" ref="A21:G22" headerRowDxfId="36" dataDxfId="35" totalsRowDxfId="34">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="site" dataDxfId="104">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="site" dataDxfId="33">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0900-000004000000}" name="brukernavn" dataDxfId="103"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0900-000005000000}" name="passord" dataDxfId="102"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0900-000003000000}" name="vty_lines" dataDxfId="101"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="secret" dataDxfId="100"/>
-    <tableColumn id="6" xr3:uid="{6E1C64EA-E908-43A5-A19B-99C374EB85DA}" name="etherchan_num" dataDxfId="99"/>
-    <tableColumn id="7" xr3:uid="{F98D4D3D-F93C-49B0-A82E-E7735EE28F3A}" name="span_port" dataDxfId="98" totalsRowDxfId="97"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0900-000004000000}" name="brukernavn" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0900-000005000000}" name="passord" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0900-000003000000}" name="vty_lines" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="secret" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{6E1C64EA-E908-43A5-A19B-99C374EB85DA}" name="etherchan_num" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{F98D4D3D-F93C-49B0-A82E-E7735EE28F3A}" name="span_port" dataDxfId="27" totalsRowDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF0B000000}" name="Tabell2" displayName="Tabell2" ref="A4:K8" headerRowDxfId="96" dataDxfId="95" totalsRowDxfId="94">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF0B000000}" name="Tabell2" displayName="Tabell2" ref="A4:K8" headerRowDxfId="25" dataDxfId="24" totalsRowDxfId="23">
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="vrf" dataDxfId="93"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="vlan" dataDxfId="92"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="interface" dataDxfId="91"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="nett id" dataDxfId="90"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="gateway" dataDxfId="89"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="mask" dataDxfId="88"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0B00-000007000000}" name="address min" dataDxfId="87"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0B00-000008000000}" name="address max" dataDxfId="86"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0B00-000009000000}" name="antall-res" dataDxfId="85"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0B00-00000A000000}" name="pri-afxx" dataDxfId="84"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0B00-00000B000000}" name="pri-1-10" dataDxfId="83"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="vrf" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="vlan" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="interface" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="nett id" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="gateway" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="mask" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0B00-000007000000}" name="address min" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0B00-000008000000}" name="address max" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0B00-000009000000}" name="antall-res" dataDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0B00-00000A000000}" name="pri-afxx" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0B00-00000B000000}" name="pri-1-10" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{F6D2D0B3-AC19-4330-8EA4-141F9D281721}" name="Tabell161824282532" displayName="Tabell161824282532" ref="A24:K25" totalsRowShown="0" headerRowDxfId="82">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="31" xr:uid="{F6D2D0B3-AC19-4330-8EA4-141F9D281721}" name="Tabell161824282532" displayName="Tabell161824282532" ref="A24:K25" totalsRowShown="0" headerRowDxfId="11">
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{560831C8-B596-49F3-902F-46F69E211EA1}" name="SW" dataDxfId="81">
+    <tableColumn id="1" xr3:uid="{560831C8-B596-49F3-902F-46F69E211EA1}" name="SW" dataDxfId="10">
       <calculatedColumnFormula>(ROW())-(ROW()-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{E82596D6-B991-40CC-95CB-F21DAE7174AF}" name="MGMT Vlan" dataDxfId="80"/>
-    <tableColumn id="3" xr3:uid="{5DE7EB2B-4947-4A2E-96FE-713844832608}" name="MGMT ip" dataDxfId="79">
+    <tableColumn id="2" xr3:uid="{E82596D6-B991-40CC-95CB-F21DAE7174AF}" name="MGMT Vlan" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{5DE7EB2B-4947-4A2E-96FE-713844832608}" name="MGMT ip" dataDxfId="8">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{96CD71AE-EBD8-4706-A140-6AC053EB9D28}" name="gateway" dataDxfId="78">
+    <tableColumn id="4" xr3:uid="{96CD71AE-EBD8-4706-A140-6AC053EB9D28}" name="gateway" dataDxfId="7">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{EB395938-8C00-462D-9B40-47A26EDC7494}" name="mask" dataDxfId="77">
+    <tableColumn id="5" xr3:uid="{EB395938-8C00-462D-9B40-47A26EDC7494}" name="mask" dataDxfId="6">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{BEB39869-24FF-4EAE-8FE0-8926AB748E68}" name="num_ports_tot" dataDxfId="76"/>
-    <tableColumn id="11" xr3:uid="{7B550E67-B906-4FBE-A432-CB0264AAA31E}" name="skiped_ports" dataDxfId="75"/>
-    <tableColumn id="6" xr3:uid="{09844D28-5E38-4CAF-946D-C86202E9AB1E}" name="num_downlink" dataDxfId="74"/>
-    <tableColumn id="7" xr3:uid="{DE656B07-9307-42AC-BAE7-A54033CC0179}" name="vlan-antall" dataDxfId="73"/>
-    <tableColumn id="8" xr3:uid="{C038B262-B22A-4F60-9F95-C1B59C71979D}" name="intf_prefix" dataDxfId="72"/>
-    <tableColumn id="9" xr3:uid="{50AA9385-3687-4437-9979-70EDBEC87403}" name="num_port_ledig" dataDxfId="71">
+    <tableColumn id="10" xr3:uid="{BEB39869-24FF-4EAE-8FE0-8926AB748E68}" name="num_ports_tot" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{7B550E67-B906-4FBE-A432-CB0264AAA31E}" name="skiped_ports" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{09844D28-5E38-4CAF-946D-C86202E9AB1E}" name="num_downlink" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{DE656B07-9307-42AC-BAE7-A54033CC0179}" name="vlan-antall" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{C038B262-B22A-4F60-9F95-C1B59C71979D}" name="intf_prefix" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{50AA9385-3687-4437-9979-70EDBEC87403}" name="num_port_ledig" dataDxfId="0">
       <calculatedColumnFormula>IF($A25=1,F25-G25-H25*$F$22-2 - IF($G$22,1,0),F25-G25-(1+H25)*$F$22-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2692,125 +2701,125 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{E77F9053-1CAC-4536-82D9-E6B1B13AB72B}" name="Tabell125" displayName="Tabell125" ref="A1:I2" headerRowDxfId="70" dataDxfId="69" totalsRowDxfId="68">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{E77F9053-1CAC-4536-82D9-E6B1B13AB72B}" name="Tabell125" displayName="Tabell125" ref="A1:I2" headerRowDxfId="164" dataDxfId="163" totalsRowDxfId="162">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{E6E46586-344C-4403-BB01-8EDB21806028}" name="site" dataDxfId="67"/>
-    <tableColumn id="2" xr3:uid="{FCB86D2F-39D7-4C90-9092-FDE5589AE525}" name="intf_prefix" dataDxfId="66"/>
-    <tableColumn id="3" xr3:uid="{4C85F93E-6153-4941-AADD-4019A25224B0}" name="router-id" dataDxfId="65">
+    <tableColumn id="1" xr3:uid="{E6E46586-344C-4403-BB01-8EDB21806028}" name="site" dataDxfId="161"/>
+    <tableColumn id="2" xr3:uid="{FCB86D2F-39D7-4C90-9092-FDE5589AE525}" name="intf_prefix" dataDxfId="160"/>
+    <tableColumn id="3" xr3:uid="{4C85F93E-6153-4941-AADD-4019A25224B0}" name="router-id" dataDxfId="159">
       <calculatedColumnFormula>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;".0"</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5628DB3F-6470-4F58-9719-CDC226F91032}" name="brukernavn" dataDxfId="64"/>
-    <tableColumn id="5" xr3:uid="{994E14D8-8E32-40DE-BC25-819473006B20}" name="passord" dataDxfId="63"/>
-    <tableColumn id="6" xr3:uid="{2510C162-2769-467E-B239-B42884D23CB5}" name="vty_lines" dataDxfId="62"/>
-    <tableColumn id="7" xr3:uid="{088B1191-63A9-47D4-9FD9-A962552749AB}" name="secret" dataDxfId="61"/>
-    <tableColumn id="8" xr3:uid="{6F304FFA-3989-4D92-B562-E9570C9F3576}" name="tacacs_key" dataDxfId="60">
+    <tableColumn id="4" xr3:uid="{5628DB3F-6470-4F58-9719-CDC226F91032}" name="brukernavn" dataDxfId="158"/>
+    <tableColumn id="5" xr3:uid="{994E14D8-8E32-40DE-BC25-819473006B20}" name="passord" dataDxfId="157"/>
+    <tableColumn id="6" xr3:uid="{2510C162-2769-467E-B239-B42884D23CB5}" name="vty_lines" dataDxfId="156"/>
+    <tableColumn id="7" xr3:uid="{088B1191-63A9-47D4-9FD9-A962552749AB}" name="secret" dataDxfId="155"/>
+    <tableColumn id="8" xr3:uid="{6F304FFA-3989-4D92-B562-E9570C9F3576}" name="tacacs_key" dataDxfId="154">
       <calculatedColumnFormula>'Site 1 (HUB)'!H2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3C3A8CE7-2167-44CF-8A83-CBF8A3913DF1}" name="dns_servers" dataDxfId="59"/>
+    <tableColumn id="9" xr3:uid="{3C3A8CE7-2167-44CF-8A83-CBF8A3913DF1}" name="dns_servers" dataDxfId="153"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{E5A2C5BB-52BB-4C1C-9F21-28A1781370B3}" name="Tabell326" displayName="Tabell326" ref="A10:D14" headerRowDxfId="58" dataDxfId="57" totalsRowDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{E5A2C5BB-52BB-4C1C-9F21-28A1781370B3}" name="Tabell326" displayName="Tabell326" ref="A11:D16" headerRowDxfId="152" dataDxfId="151" totalsRowDxfId="150">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{CF7349DE-C31B-4FC6-83C6-8B6628474834}" name="vrf" dataDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{F73FC7A9-205A-4D8C-8765-0C403F93088B}" name="rt" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{53625FDA-B6AB-45DC-B3A1-11B9F3FB71ED}" name="loopback" dataDxfId="54"/>
-    <tableColumn id="4" xr3:uid="{E89555BA-5F3F-4C0B-9EB1-2E878627A098}" name="laddr" dataDxfId="53"/>
+    <tableColumn id="1" xr3:uid="{CF7349DE-C31B-4FC6-83C6-8B6628474834}" name="vrf" dataDxfId="149"/>
+    <tableColumn id="2" xr3:uid="{F73FC7A9-205A-4D8C-8765-0C403F93088B}" name="rt" dataDxfId="148"/>
+    <tableColumn id="3" xr3:uid="{53625FDA-B6AB-45DC-B3A1-11B9F3FB71ED}" name="loopback" dataDxfId="147"/>
+    <tableColumn id="4" xr3:uid="{E89555BA-5F3F-4C0B-9EB1-2E878627A098}" name="laddr" dataDxfId="146"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{65A662B1-EB00-41C5-9AA3-10F1A1AB2E06}" name="Tabell427" displayName="Tabell427" ref="A16:J19" headerRowDxfId="52" dataDxfId="51" totalsRowDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{65A662B1-EB00-41C5-9AA3-10F1A1AB2E06}" name="Tabell427" displayName="Tabell427" ref="A18:J21" headerRowDxfId="145" dataDxfId="144" totalsRowDxfId="143">
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{2ECB4295-60F9-49EA-9455-A3D81A24F7A0}" name="tunnel id" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{13A72EC2-1D8A-4222-BD41-BE2592A960A7}" name="vrf" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{223D8914-883F-4017-82DA-E5AB71951DF9}" name="ip address" dataDxfId="47">
-      <calculatedColumnFormula>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H17+$A$2)</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{2ECB4295-60F9-49EA-9455-A3D81A24F7A0}" name="tunnel id" dataDxfId="142"/>
+    <tableColumn id="2" xr3:uid="{13A72EC2-1D8A-4222-BD41-BE2592A960A7}" name="vrf" dataDxfId="141"/>
+    <tableColumn id="3" xr3:uid="{223D8914-883F-4017-82DA-E5AB71951DF9}" name="ip address" dataDxfId="140">
+      <calculatedColumnFormula>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H19+$A$2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{24341D21-5A53-49ED-81C2-4F808B523A33}" name="mask" dataDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{B6651250-1C15-4916-9DD5-0DECA970E8E7}" name="source" dataDxfId="45">
+    <tableColumn id="4" xr3:uid="{24341D21-5A53-49ED-81C2-4F808B523A33}" name="mask" dataDxfId="139"/>
+    <tableColumn id="5" xr3:uid="{B6651250-1C15-4916-9DD5-0DECA970E8E7}" name="source" dataDxfId="138">
       <calculatedColumnFormula>$C$2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{8B863BC6-A759-4605-BC9F-50C3CABE8006}" name="destination" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{BF23358A-67B7-45E8-AFF4-D27FC9289BE3}" name="gre mode" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{C26012CA-6896-40EB-BAB9-E2B7AC017DAF}" name="network-id" dataDxfId="42"/>
-    <tableColumn id="9" xr3:uid="{D286B9CB-857F-4868-8DE1-FD5BECC2B334}" name="ipsec" dataDxfId="41"/>
-    <tableColumn id="10" xr3:uid="{293E9FC5-D0E5-407D-A659-65944E4EA279}" name="ipsec key" dataDxfId="40"/>
+    <tableColumn id="6" xr3:uid="{8B863BC6-A759-4605-BC9F-50C3CABE8006}" name="destination" dataDxfId="137"/>
+    <tableColumn id="7" xr3:uid="{BF23358A-67B7-45E8-AFF4-D27FC9289BE3}" name="gre mode" dataDxfId="136"/>
+    <tableColumn id="8" xr3:uid="{C26012CA-6896-40EB-BAB9-E2B7AC017DAF}" name="network-id" dataDxfId="135"/>
+    <tableColumn id="9" xr3:uid="{D286B9CB-857F-4868-8DE1-FD5BECC2B334}" name="ipsec" dataDxfId="134"/>
+    <tableColumn id="10" xr3:uid="{293E9FC5-D0E5-407D-A659-65944E4EA279}" name="ipsec key" dataDxfId="133"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{1E2C2B46-26EF-4E8A-BF33-BE80A9579C3A}" name="Tabell1319253028" displayName="Tabell1319253028" ref="A21:G22" headerRowDxfId="39" dataDxfId="38" totalsRowDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{1E2C2B46-26EF-4E8A-BF33-BE80A9579C3A}" name="Tabell1319253028" displayName="Tabell1319253028" ref="A23:G24" headerRowDxfId="132" dataDxfId="131" totalsRowDxfId="130">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{DA701FF9-2640-4ED3-9CA5-2E83863ECACD}" name="site" dataDxfId="36">
+    <tableColumn id="1" xr3:uid="{DA701FF9-2640-4ED3-9CA5-2E83863ECACD}" name="site" dataDxfId="129">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{A0A92227-4ED4-45A6-AF74-08CAD53943A6}" name="brukernavn" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{760D6751-0B3C-4CD1-BBA0-61B78451CA09}" name="passord" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{EFF5613C-F01D-4E28-95CD-C69E310DD62B}" name="vty_lines" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{2102378C-EB85-46A2-AACC-F9D8E8BE9DD6}" name="secret" dataDxfId="32"/>
-    <tableColumn id="6" xr3:uid="{B5B5EDC5-D203-4FAB-BF0C-B091D363D2A5}" name="etherchan_num" dataDxfId="31"/>
-    <tableColumn id="7" xr3:uid="{EEE8114C-5818-4125-AFC9-23640FDD8FDB}" name="span_port" dataDxfId="30" totalsRowDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{A0A92227-4ED4-45A6-AF74-08CAD53943A6}" name="brukernavn" dataDxfId="128"/>
+    <tableColumn id="5" xr3:uid="{760D6751-0B3C-4CD1-BBA0-61B78451CA09}" name="passord" dataDxfId="127"/>
+    <tableColumn id="3" xr3:uid="{EFF5613C-F01D-4E28-95CD-C69E310DD62B}" name="vty_lines" dataDxfId="126"/>
+    <tableColumn id="2" xr3:uid="{2102378C-EB85-46A2-AACC-F9D8E8BE9DD6}" name="secret" dataDxfId="125"/>
+    <tableColumn id="6" xr3:uid="{B5B5EDC5-D203-4FAB-BF0C-B091D363D2A5}" name="etherchan_num" dataDxfId="124"/>
+    <tableColumn id="7" xr3:uid="{EEE8114C-5818-4125-AFC9-23640FDD8FDB}" name="span_port" dataDxfId="123" totalsRowDxfId="122"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{769C0F37-0A83-420D-A8E1-9EE1313312AC}" name="Tabell231" displayName="Tabell231" ref="A4:K8" headerRowDxfId="28" dataDxfId="27" totalsRowDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="30" xr:uid="{769C0F37-0A83-420D-A8E1-9EE1313312AC}" name="Tabell231" displayName="Tabell231" ref="A4:K9" headerRowDxfId="121" dataDxfId="120" totalsRowDxfId="119">
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{B8E867F1-3F4C-41D0-86F6-FE265CF06F61}" name="vrf" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{D18AC450-DB0E-4854-A38A-3EB64C6DD4EB}" name="vlan" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{95B88648-5211-4200-988D-51B7D899A2BF}" name="interface" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{341E7F84-C497-477E-9951-D8B1F0235F22}" name="nett id" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{21C6E08A-5925-4A18-B96B-DC4B4117EAD0}" name="gateway" dataDxfId="21">
+    <tableColumn id="1" xr3:uid="{B8E867F1-3F4C-41D0-86F6-FE265CF06F61}" name="vrf" dataDxfId="118"/>
+    <tableColumn id="2" xr3:uid="{D18AC450-DB0E-4854-A38A-3EB64C6DD4EB}" name="vlan" dataDxfId="117"/>
+    <tableColumn id="3" xr3:uid="{95B88648-5211-4200-988D-51B7D899A2BF}" name="interface" dataDxfId="116"/>
+    <tableColumn id="4" xr3:uid="{341E7F84-C497-477E-9951-D8B1F0235F22}" name="nett id" dataDxfId="115"/>
+    <tableColumn id="5" xr3:uid="{21C6E08A-5925-4A18-B96B-DC4B4117EAD0}" name="gateway" dataDxfId="114">
       <calculatedColumnFormula>LEFT(D5,LEN(D5)-1)&amp;"1"</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{16980205-5AE1-4CAF-9B95-493327E6B6C3}" name="mask" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{4660DC90-F49A-4202-BD4B-71BC6584979A}" name="address min" dataDxfId="19">
+    <tableColumn id="6" xr3:uid="{16980205-5AE1-4CAF-9B95-493327E6B6C3}" name="mask" dataDxfId="113"/>
+    <tableColumn id="7" xr3:uid="{4660DC90-F49A-4202-BD4B-71BC6584979A}" name="address min" dataDxfId="112">
       <calculatedColumnFormula>LEFT(D5,LEN(D5)-1)&amp;"1"</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{ADA93C1E-2F32-478C-AA86-4FC2ED08742C}" name="address max" dataDxfId="18">
+    <tableColumn id="8" xr3:uid="{ADA93C1E-2F32-478C-AA86-4FC2ED08742C}" name="address max" dataDxfId="111">
       <calculatedColumnFormula>LEFT(D5,FIND(".",D5,FIND(".",D5)+1)-1)&amp;".255.254"</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{CA8441FD-37D1-4117-91A7-FA904F322160}" name="antall-res" dataDxfId="17"/>
-    <tableColumn id="10" xr3:uid="{1F6500D8-8B23-4118-A326-933F33A88F27}" name="pri-afxx" dataDxfId="16"/>
-    <tableColumn id="11" xr3:uid="{AC9A4C9B-1C06-4728-8D9C-E07A015E6BCA}" name="pri-1-10" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{CA8441FD-37D1-4117-91A7-FA904F322160}" name="antall-res" dataDxfId="110"/>
+    <tableColumn id="10" xr3:uid="{1F6500D8-8B23-4118-A326-933F33A88F27}" name="pri-afxx" dataDxfId="109"/>
+    <tableColumn id="11" xr3:uid="{AC9A4C9B-1C06-4728-8D9C-E07A015E6BCA}" name="pri-1-10" dataDxfId="108"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{CEC4A60A-F98B-45B0-B6EF-F3AF53EA1619}" name="Tabell16182428253233" displayName="Tabell16182428253233" ref="A24:K25" totalsRowShown="0" headerRowDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="32" xr:uid="{CEC4A60A-F98B-45B0-B6EF-F3AF53EA1619}" name="Tabell16182428253233" displayName="Tabell16182428253233" ref="A26:K27" totalsRowShown="0" headerRowDxfId="107">
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4102DBA8-76EC-46C2-97AC-C45CCA6C3959}" name="SW" dataDxfId="13">
+    <tableColumn id="1" xr3:uid="{4102DBA8-76EC-46C2-97AC-C45CCA6C3959}" name="SW" dataDxfId="106">
       <calculatedColumnFormula>(ROW())-(ROW()-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{88524807-430F-4F05-A66A-A026753796D8}" name="MGMT Vlan" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{AC8B28E6-E5DC-45AE-BE1C-4C52D8077002}" name="MGMT ip" dataDxfId="11">
-      <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</calculatedColumnFormula>
+    <tableColumn id="2" xr3:uid="{88524807-430F-4F05-A66A-A026753796D8}" name="MGMT Vlan" dataDxfId="105"/>
+    <tableColumn id="3" xr3:uid="{AC8B28E6-E5DC-45AE-BE1C-4C52D8077002}" name="MGMT ip" dataDxfId="104">
+      <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A27)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{07AB9192-8CD5-4149-8F18-77D5ACBE4F9E}" name="gateway" dataDxfId="10">
+    <tableColumn id="4" xr3:uid="{07AB9192-8CD5-4149-8F18-77D5ACBE4F9E}" name="gateway" dataDxfId="103">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{D5DA3E60-36DA-4C88-88FF-10FDD9C14A18}" name="mask" dataDxfId="9">
+    <tableColumn id="5" xr3:uid="{D5DA3E60-36DA-4C88-88FF-10FDD9C14A18}" name="mask" dataDxfId="102">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{4E3337F9-025D-4DA0-982C-3E70497F895A}" name="num_ports_tot" dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{647707FF-22D1-4F6D-A670-EDBB67D47D4B}" name="skiped_ports" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{BE2F1799-FA72-40F2-9D10-AF25AC3BCF6E}" name="num_downlink" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{E6B5A026-07C4-4081-84E5-F4A83023F33C}" name="vlan-antall" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{88056F0E-CDA4-4FC7-B241-EE7FA7CD666F}" name="intf_prefix" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{016D87AC-4D94-4EDA-B2B6-4B3887442A16}" name="num_port_ledig" dataDxfId="3">
-      <calculatedColumnFormula>IF($A25=1,F25-G25-H25*$F$22-2 - IF($G$22,1,0),F25-G25-(1+H25)*$F$22-1)</calculatedColumnFormula>
+    <tableColumn id="10" xr3:uid="{4E3337F9-025D-4DA0-982C-3E70497F895A}" name="num_ports_tot" dataDxfId="101"/>
+    <tableColumn id="11" xr3:uid="{647707FF-22D1-4F6D-A670-EDBB67D47D4B}" name="skiped_ports" dataDxfId="100"/>
+    <tableColumn id="6" xr3:uid="{BE2F1799-FA72-40F2-9D10-AF25AC3BCF6E}" name="num_downlink" dataDxfId="99"/>
+    <tableColumn id="7" xr3:uid="{E6B5A026-07C4-4081-84E5-F4A83023F33C}" name="vlan-antall" dataDxfId="98"/>
+    <tableColumn id="8" xr3:uid="{88056F0E-CDA4-4FC7-B241-EE7FA7CD666F}" name="intf_prefix" dataDxfId="97"/>
+    <tableColumn id="9" xr3:uid="{016D87AC-4D94-4EDA-B2B6-4B3887442A16}" name="num_port_ledig" dataDxfId="96">
+      <calculatedColumnFormula>IF($A27=1,F27-G27-H27*$F$24-2 - IF($G$24,1,0),F27-G27-(1+H27)*$F$24-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
@@ -2828,7 +2837,7 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="mask"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="address min"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="address max"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="antall-res" dataDxfId="160"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="antall-res" dataDxfId="91"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0100-00000A000000}" name="pri-afxx"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0100-00000B000000}" name="pri-1-10"/>
   </tableColumns>
@@ -2840,7 +2849,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabell7" displayName="Tabell7" ref="A10:D14">
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="vrf"/>
-    <tableColumn id="2" xr3:uid="{84DE2886-BEBC-478D-A126-1D1701C2FABA}" name="rt" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{84DE2886-BEBC-478D-A126-1D1701C2FABA}" name="rt" dataDxfId="90"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="loopback"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="laddr">
       <calculatedColumnFormula>$A$2&amp;"."&amp;$A$2&amp;"."&amp;$A$2&amp;"."&amp;(C11)</calculatedColumnFormula>
@@ -2859,7 +2868,7 @@
       <calculatedColumnFormula>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H17+$A$2)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="mask"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="source" dataDxfId="159">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="source" dataDxfId="89">
       <calculatedColumnFormula>$C$2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="destination"/>
@@ -2873,44 +2882,44 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabell131921" displayName="Tabell131921" ref="A21:G22" dataDxfId="158">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabell131921" displayName="Tabell131921" ref="A21:G22" dataDxfId="88">
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="site" dataDxfId="157">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="site" dataDxfId="87">
       <calculatedColumnFormula>A2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="brukernavn" dataDxfId="156"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="passord" dataDxfId="155"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="vty_lines" dataDxfId="154"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="secret" dataDxfId="153"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="etherchan_num" dataDxfId="152"/>
-    <tableColumn id="7" xr3:uid="{2F89DC28-B462-4A4B-9338-E6327171D3B6}" name="span_port" dataDxfId="151"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="brukernavn" dataDxfId="86"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="passord" dataDxfId="85"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="vty_lines" dataDxfId="84"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="secret" dataDxfId="83"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0400-000006000000}" name="etherchan_num" dataDxfId="82"/>
+    <tableColumn id="7" xr3:uid="{2F89DC28-B462-4A4B-9338-E6327171D3B6}" name="span_port" dataDxfId="81"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Tabell1618242825" displayName="Tabell1618242825" ref="A24:K26" totalsRowShown="0" headerRowDxfId="150">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Tabell1618242825" displayName="Tabell1618242825" ref="A24:K26" totalsRowShown="0" headerRowDxfId="80">
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="SW" dataDxfId="149">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="SW" dataDxfId="79">
       <calculatedColumnFormula>(ROW())-(ROW()-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="MGMT Vlan" dataDxfId="148"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="MGMT ip" dataDxfId="147">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="MGMT Vlan" dataDxfId="78"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="MGMT ip" dataDxfId="77">
       <calculatedColumnFormula>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="gateway" dataDxfId="146">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="gateway" dataDxfId="76">
       <calculatedColumnFormula>$E$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="mask" dataDxfId="145">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="mask" dataDxfId="75">
       <calculatedColumnFormula>$F$5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" name="num_ports_tot" dataDxfId="144"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0500-00000B000000}" name="skiped_ports" dataDxfId="143"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="num_downlink" dataDxfId="142"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="vlan-antall" dataDxfId="141"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="intf_prefix" dataDxfId="140"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="num_port_ledig" dataDxfId="139">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" name="num_ports_tot" dataDxfId="74"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0500-00000B000000}" name="skiped_ports" dataDxfId="73"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="num_downlink" dataDxfId="72"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="vlan-antall" dataDxfId="71"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="intf_prefix" dataDxfId="70"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="num_port_ledig" dataDxfId="69">
       <calculatedColumnFormula>IF($A25=1,F25-G25-H25*$F$22-2 - IF($G$22,1,0),F25-G25-(1+H25)*$F$22-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2919,53 +2928,53 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Tabell1" displayName="Tabell1" ref="A1:I2" headerRowDxfId="138" dataDxfId="137" totalsRowDxfId="136">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="Tabell1" displayName="Tabell1" ref="A1:I2" headerRowDxfId="68" dataDxfId="67" totalsRowDxfId="66">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="site" dataDxfId="135"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="intf_prefix" dataDxfId="134"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="router-id" dataDxfId="133"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="brukernavn" dataDxfId="132"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="passord" dataDxfId="131"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="vty_lines" dataDxfId="130"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="secret" dataDxfId="129"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" name="tacacs_key" dataDxfId="128">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="site" dataDxfId="65"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="intf_prefix" dataDxfId="64"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="router-id" dataDxfId="63"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="brukernavn" dataDxfId="62"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="passord" dataDxfId="61"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="vty_lines" dataDxfId="60"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="secret" dataDxfId="59"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" name="tacacs_key" dataDxfId="58">
       <calculatedColumnFormula>'Site 1 (HUB)'!H2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A5DE2194-7404-46E4-B6C2-ABF2C830FF23}" name="dns_servers" dataDxfId="127"/>
+    <tableColumn id="9" xr3:uid="{A5DE2194-7404-46E4-B6C2-ABF2C830FF23}" name="dns_servers" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="Tabell3" displayName="Tabell3" ref="A10:D14" headerRowDxfId="126" dataDxfId="125" totalsRowDxfId="124">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="Tabell3" displayName="Tabell3" ref="A10:D14" headerRowDxfId="56" dataDxfId="55" totalsRowDxfId="54">
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="vrf" dataDxfId="123"/>
-    <tableColumn id="2" xr3:uid="{073AEF7E-35F4-47BE-A04E-55474C09C0B3}" name="rt" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="loopback" dataDxfId="122"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="laddr" dataDxfId="121"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="vrf" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{073AEF7E-35F4-47BE-A04E-55474C09C0B3}" name="rt" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="loopback" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="laddr" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Tabell4" displayName="Tabell4" ref="A16:J19" headerRowDxfId="120" dataDxfId="119" totalsRowDxfId="118">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{00000000-000C-0000-FFFF-FFFF08000000}" name="Tabell4" displayName="Tabell4" ref="A16:J19" headerRowDxfId="49" dataDxfId="48" totalsRowDxfId="47">
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="tunnel id" dataDxfId="117"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="vrf" dataDxfId="116"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="ip address" dataDxfId="115">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0800-000001000000}" name="tunnel id" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0800-000002000000}" name="vrf" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="ip address" dataDxfId="44">
       <calculatedColumnFormula>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H17+$A$2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="mask" dataDxfId="114"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="source" dataDxfId="113">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="mask" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="source" dataDxfId="42">
       <calculatedColumnFormula>$C$2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="destination" dataDxfId="112"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="gre mode" dataDxfId="111"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0800-000008000000}" name="network-id" dataDxfId="110"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0800-000009000000}" name="ipsec" dataDxfId="109"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0800-00000A000000}" name="ipsec key" dataDxfId="108"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="destination" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="gre mode" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0800-000008000000}" name="network-id" dataDxfId="39"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0800-000009000000}" name="ipsec" dataDxfId="38"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0800-00000A000000}" name="ipsec key" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6390,7 +6399,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -6675,31 +6684,49 @@
       </c>
     </row>
     <row r="9" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="14"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="14"/>
+      <c r="A9" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="14">
+        <v>50</v>
+      </c>
+      <c r="C9" s="14">
+        <v>0</v>
+      </c>
+      <c r="D9" s="14" t="str">
+        <f>10&amp;"."&amp;(B9+A3)&amp;"."&amp;0&amp;"."&amp;0</f>
+        <v>10.50.0.0</v>
+      </c>
+      <c r="E9" s="14" t="str">
+        <f t="shared" ref="E9" si="2">LEFT(D9,LEN(D9)-1)&amp;"1"</f>
+        <v>10.50.0.1</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="G9" s="14" t="str">
+        <f t="shared" ref="G9" si="3">LEFT(D9,LEN(D9)-1)&amp;"1"</f>
+        <v>10.50.0.1</v>
+      </c>
+      <c r="H9" s="14" t="str">
+        <f>LEFT(D9,FIND(".",D9,FIND(".",D9)+1)-1)&amp;".255.254"</f>
+        <v>10.50.255.254</v>
+      </c>
+      <c r="I9" s="14">
+        <v>10</v>
+      </c>
+      <c r="J9" s="14">
+        <v>41</v>
+      </c>
+      <c r="K9" s="14">
+        <v>10</v>
+      </c>
     </row>
-    <row r="10" spans="1:12" ht="15" x14ac:dyDescent="0.2">
-      <c r="A10" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>31</v>
-      </c>
+    <row r="10" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
       <c r="E10" s="14"/>
       <c r="F10" s="14"/>
       <c r="G10" s="14"/>
@@ -6707,21 +6734,19 @@
       <c r="I10" s="14"/>
       <c r="J10" s="14"/>
       <c r="K10" s="14"/>
-      <c r="L10" s="14"/>
     </row>
-    <row r="11" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="C11" s="14">
-        <v>10</v>
-      </c>
-      <c r="D11" s="14" t="str">
-        <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;(C11)</f>
-        <v>3.3.3.10</v>
+        <v>14</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>31</v>
       </c>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
@@ -6734,17 +6759,17 @@
     </row>
     <row r="12" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C12" s="14">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D12" s="14" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;(C12)</f>
-        <v>3.3.3.20</v>
+        <v>3.3.3.10</v>
       </c>
       <c r="E12" s="14"/>
       <c r="F12" s="14"/>
@@ -6757,17 +6782,17 @@
     </row>
     <row r="13" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A13" s="14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C13" s="14">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D13" s="14" t="str">
         <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;(C13)</f>
-        <v>3.3.3.30</v>
+        <v>3.3.3.20</v>
       </c>
       <c r="E13" s="14"/>
       <c r="F13" s="14"/>
@@ -6780,17 +6805,17 @@
     </row>
     <row r="14" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C14" s="14">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D14" s="14" t="str">
-        <f t="shared" ref="D14" si="2">$A$2&amp;"."&amp;$A$2&amp;"."&amp;$A$2&amp;"."&amp;(C14)</f>
-        <v>3.3.3.40</v>
+        <f>A2&amp;"."&amp;A2&amp;"."&amp;A2&amp;"."&amp;(C14)</f>
+        <v>3.3.3.30</v>
       </c>
       <c r="E14" s="14"/>
       <c r="F14" s="14"/>
@@ -6802,10 +6827,19 @@
       <c r="L14" s="14"/>
     </row>
     <row r="15" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
+      <c r="A15" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="14">
+        <v>40</v>
+      </c>
+      <c r="D15" s="14" t="str">
+        <f t="shared" ref="D15" si="4">$A$2&amp;"."&amp;$A$2&amp;"."&amp;$A$2&amp;"."&amp;(C15)</f>
+        <v>3.3.3.40</v>
+      </c>
       <c r="E15" s="14"/>
       <c r="F15" s="14"/>
       <c r="G15" s="14"/>
@@ -6813,120 +6847,93 @@
       <c r="I15" s="14"/>
       <c r="J15" s="14"/>
       <c r="K15" s="14"/>
+      <c r="L15" s="14"/>
     </row>
     <row r="16" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A16" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="G16" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="H16" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="I16" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="J16" s="14" t="s">
-        <v>39</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="14">
+        <v>50</v>
+      </c>
+      <c r="D16" s="14" t="str">
+        <f t="shared" ref="D16" si="5">$A$2&amp;"."&amp;$A$2&amp;"."&amp;$A$2&amp;"."&amp;(C16)</f>
+        <v>3.3.3.50</v>
+      </c>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+      <c r="G16" s="14"/>
+      <c r="H16" s="14"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
       <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
     </row>
     <row r="17" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="14" t="str">
-        <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H17+$A$2)</f>
-        <v>172.16.0.13</v>
-      </c>
-      <c r="D17" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="E17" s="14" t="str">
-        <f t="shared" ref="E17:E19" si="3">$C$2</f>
-        <v>3.3.3.0</v>
-      </c>
+      <c r="A17" s="14"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
       <c r="F17" s="14"/>
-      <c r="G17" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="H17" s="14">
-        <v>10</v>
-      </c>
-      <c r="I17" s="14">
-        <f t="array" ref="I17">'Site 1 (HUB)'!I17</f>
-        <v>0</v>
-      </c>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="14"/>
       <c r="J17" s="14"/>
       <c r="K17" s="14"/>
     </row>
     <row r="18" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" s="14" t="str">
-        <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H18+$A$2)</f>
-        <v>172.16.0.33</v>
+        <v>14</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>33</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="E18" s="14" t="str">
-        <f t="shared" si="3"/>
-        <v>3.3.3.0</v>
-      </c>
-      <c r="F18" s="14"/>
+        <v>19</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>35</v>
+      </c>
       <c r="G18" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="H18" s="14">
-        <v>30</v>
-      </c>
-      <c r="I18" s="14" t="b">
-        <f t="array" ref="I18">'Site 1 (HUB)'!I18</f>
-        <v>1</v>
-      </c>
-      <c r="J18" s="14"/>
+        <v>36</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="I18" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="J18" s="14" t="s">
+        <v>39</v>
+      </c>
       <c r="K18" s="14"/>
     </row>
     <row r="19" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A19" s="14" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C19" s="14" t="str">
-        <f t="shared" ref="C19" si="4">172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H19+$A$2)</f>
-        <v>172.16.0.43</v>
+        <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H19+$A$2)</f>
+        <v>172.16.0.13</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>41</v>
       </c>
       <c r="E19" s="14" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="E19:E21" si="6">$C$2</f>
         <v>3.3.3.0</v>
       </c>
       <c r="F19" s="14"/>
@@ -6934,188 +6941,252 @@
         <v>42</v>
       </c>
       <c r="H19" s="14">
-        <v>40</v>
-      </c>
-      <c r="I19" s="14" t="b">
-        <f>'Site 1 (HUB)'!I19</f>
-        <v>1</v>
+        <v>10</v>
+      </c>
+      <c r="I19" s="14">
+        <f t="array" ref="I19">'Site 1 (HUB)'!I17</f>
+        <v>0</v>
       </c>
       <c r="J19" s="14"/>
       <c r="K19" s="14"/>
     </row>
     <row r="20" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A20" s="14"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
+      <c r="A20" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" s="14" t="str">
+        <f>172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H20+$A$2)</f>
+        <v>172.16.0.33</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>3.3.3.0</v>
+      </c>
       <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
+      <c r="G20" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="H20" s="14">
+        <v>30</v>
+      </c>
+      <c r="I20" s="14" t="b">
+        <f t="array" ref="I20">'Site 1 (HUB)'!I18</f>
+        <v>1</v>
+      </c>
       <c r="J20" s="14"/>
       <c r="K20" s="14"/>
     </row>
     <row r="21" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A21" s="14" t="s">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>4</v>
+        <v>29</v>
+      </c>
+      <c r="C21" s="14" t="str">
+        <f t="shared" ref="C21" si="7">172&amp;"."&amp;16&amp;"."&amp;0&amp;"."&amp;(H21+$A$2)</f>
+        <v>172.16.0.43</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="F21" s="14" t="s">
-        <v>56</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="E21" s="14" t="str">
+        <f t="shared" si="6"/>
+        <v>3.3.3.0</v>
+      </c>
+      <c r="F21" s="14"/>
       <c r="G21" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="H21" s="14"/>
-      <c r="I21" s="14"/>
+        <v>42</v>
+      </c>
+      <c r="H21" s="14">
+        <v>40</v>
+      </c>
+      <c r="I21" s="14" t="b">
+        <f>'Site 1 (HUB)'!I19</f>
+        <v>1</v>
+      </c>
       <c r="J21" s="14"/>
       <c r="K21" s="14"/>
     </row>
     <row r="22" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A22" s="14">
-        <f>A2</f>
-        <v>3</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="E22" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" s="14">
-        <v>2</v>
-      </c>
-      <c r="G22" s="14" t="b">
-        <v>1</v>
-      </c>
+      <c r="A22" s="14"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
       <c r="H22" s="14"/>
       <c r="I22" s="14"/>
       <c r="J22" s="14"/>
       <c r="K22" s="14"/>
     </row>
     <row r="23" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A23" s="14"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
+      <c r="A23" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="G23" s="14" t="s">
+        <v>57</v>
+      </c>
       <c r="H23" s="14"/>
       <c r="I23" s="14"/>
       <c r="J23" s="14"/>
       <c r="K23" s="14"/>
     </row>
-    <row r="24" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A24" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="F24" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="G24" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="H24" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="I24" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="J24" s="15" t="s">
+    <row r="24" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A24" s="14">
+        <f>A2</f>
+        <v>3</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="14">
+        <v>2</v>
+      </c>
+      <c r="G24" s="14" t="b">
         <v>1</v>
       </c>
-      <c r="K24" s="15" t="s">
-        <v>52</v>
-      </c>
+      <c r="H24" s="14"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="14"/>
     </row>
     <row r="25" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A25" s="8">
+      <c r="A25" s="14"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="14"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="14"/>
+    </row>
+    <row r="26" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+      <c r="A26" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G26" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="H26" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="I26" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="J26" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="K26" s="15" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A27" s="8">
         <f>(ROW())-(ROW()-1)</f>
         <v>1</v>
       </c>
-      <c r="B25" s="8">
+      <c r="B27" s="8">
         <v>10</v>
       </c>
-      <c r="C25" s="8" t="str">
-        <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A25)</f>
+      <c r="C27" s="8" t="str">
+        <f>LEFT($G$5,LEN($G$5)-1)&amp;(RIGHT($G$5,1)+A27)</f>
         <v>10.13.0.2</v>
       </c>
-      <c r="D25" s="8" t="str">
+      <c r="D27" s="8" t="str">
         <f>$E$5</f>
         <v>10.13.0.1</v>
       </c>
-      <c r="E25" s="8" t="str">
+      <c r="E27" s="8" t="str">
         <f>$F$5</f>
         <v>255.255.0.0</v>
       </c>
-      <c r="F25" s="8">
+      <c r="F27" s="8">
         <v>24</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G27" s="8">
         <v>1</v>
       </c>
-      <c r="H25" s="11">
+      <c r="H27" s="11">
         <v>0</v>
       </c>
-      <c r="I25" s="8" t="s">
+      <c r="I27" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="J25" s="2" t="s">
+      <c r="J27" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K25" s="2">
-        <f>IF($A25=1,F25-G25-H25*$F$22-2 - IF($G$22,1,0),F25-G25-(1+H25)*$F$22-1)</f>
+      <c r="K27" s="2">
+        <f>IF($A27=1,F27-G27-H27*$F$24-2 - IF($G$24,1,0),F27-G27-(1+H27)*$F$24-1)</f>
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="14"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="14"/>
-      <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
+    <row r="28" spans="1:11" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A28" s="14"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="14"/>
+      <c r="J28" s="14"/>
+      <c r="K28" s="14"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I25" xr:uid="{44077420-E806-44F5-BB6E-60A45CE71946}">
-      <formula1>IF(I25="",TRUE,SUM(--_xlfn.TEXTAFTER(_xlfn.TEXTSPLIT(I25,"-"),"."))&lt;=K25)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I27" xr:uid="{44077420-E806-44F5-BB6E-60A45CE71946}">
+      <formula1>IF(I27="",TRUE,SUM(--_xlfn.TEXTAFTER(_xlfn.TEXTSPLIT(I27,"-"),"."))&lt;=K27)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>